<commit_message>
correct pathfinerd scenario group
</commit_message>
<xml_diff>
--- a/data/dimensions/dimensions.xlsx
+++ b/data/dimensions/dimensions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jan/git/data_model_tmp/data/dimensions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2421DD3-7B23-2649-BD12-8E549041BD07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74AE55F5-5A64-214C-9C93-57475E4742C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="620" windowWidth="27520" windowHeight="22440" tabRatio="808" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="27520" windowHeight="18980" tabRatio="808" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="21" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3010" uniqueCount="1677">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3010" uniqueCount="1674">
   <si>
     <t>id</t>
   </si>
@@ -5027,9 +5027,6 @@
     <t>hpflex</t>
   </si>
   <si>
-    <t>pathfndr-sr6</t>
-  </si>
-  <si>
     <t>hpflex-no-exp</t>
   </si>
   <si>
@@ -5039,9 +5036,6 @@
     <t>noflex</t>
   </si>
   <si>
-    <t>pathfndr-sr7</t>
-  </si>
-  <si>
     <t>noflex-no-exp</t>
   </si>
   <si>
@@ -5049,9 +5043,6 @@
   </si>
   <si>
     <t>bothflex</t>
-  </si>
-  <si>
-    <t>pathfndr-sr8</t>
   </si>
   <si>
     <t>bothflex-no-exp</t>
@@ -5091,7 +5082,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5161,6 +5152,12 @@
       <color rgb="FFA5D6FF"/>
       <name val="Menlo"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -16050,50 +16047,50 @@
         <v>1656</v>
       </c>
       <c r="B75" t="s">
-        <v>1657</v>
+        <v>1652</v>
       </c>
       <c r="C75" t="s">
         <v>1653</v>
       </c>
       <c r="D75" t="s">
+        <v>1657</v>
+      </c>
+      <c r="E75" t="s">
         <v>1658</v>
-      </c>
-      <c r="E75" t="s">
-        <v>1659</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>1660</v>
+        <v>1659</v>
       </c>
       <c r="B76" t="s">
-        <v>1661</v>
+        <v>1652</v>
       </c>
       <c r="C76" t="s">
         <v>1653</v>
       </c>
       <c r="D76" t="s">
-        <v>1662</v>
+        <v>1660</v>
       </c>
       <c r="E76" t="s">
-        <v>1663</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>1664</v>
+        <v>1662</v>
       </c>
       <c r="B77" t="s">
-        <v>1665</v>
+        <v>1652</v>
       </c>
       <c r="C77" t="s">
         <v>1653</v>
       </c>
       <c r="D77" t="s">
-        <v>1666</v>
+        <v>1663</v>
       </c>
       <c r="E77" t="s">
-        <v>1667</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
@@ -16104,13 +16101,13 @@
         <v>1652</v>
       </c>
       <c r="C78" t="s">
-        <v>1668</v>
+        <v>1665</v>
       </c>
       <c r="D78" t="s">
-        <v>1669</v>
+        <v>1666</v>
       </c>
       <c r="E78" t="s">
-        <v>1670</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
@@ -16118,53 +16115,54 @@
         <v>1656</v>
       </c>
       <c r="B79" t="s">
-        <v>1657</v>
+        <v>1652</v>
       </c>
       <c r="C79" t="s">
+        <v>1665</v>
+      </c>
+      <c r="D79" t="s">
         <v>1668</v>
       </c>
-      <c r="D79" t="s">
-        <v>1671</v>
-      </c>
       <c r="E79" t="s">
-        <v>1672</v>
+        <v>1669</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>1660</v>
+        <v>1659</v>
       </c>
       <c r="B80" t="s">
-        <v>1661</v>
+        <v>1652</v>
       </c>
       <c r="C80" t="s">
-        <v>1668</v>
+        <v>1665</v>
       </c>
       <c r="D80" t="s">
-        <v>1673</v>
+        <v>1670</v>
       </c>
       <c r="E80" t="s">
-        <v>1674</v>
+        <v>1671</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>1664</v>
+        <v>1662</v>
       </c>
       <c r="B81" t="s">
+        <v>1652</v>
+      </c>
+      <c r="C81" t="s">
         <v>1665</v>
       </c>
-      <c r="C81" t="s">
-        <v>1668</v>
-      </c>
       <c r="D81" t="s">
-        <v>1675</v>
+        <v>1672</v>
       </c>
       <c r="E81" t="s">
-        <v>1676</v>
+        <v>1673</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
correct pathfinerd scenario group (#19)
</commit_message>
<xml_diff>
--- a/data/dimensions/dimensions.xlsx
+++ b/data/dimensions/dimensions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jan/git/data_model_tmp/data/dimensions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2421DD3-7B23-2649-BD12-8E549041BD07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74AE55F5-5A64-214C-9C93-57475E4742C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="620" windowWidth="27520" windowHeight="22440" tabRatio="808" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="27520" windowHeight="18980" tabRatio="808" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="21" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3010" uniqueCount="1677">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3010" uniqueCount="1674">
   <si>
     <t>id</t>
   </si>
@@ -5027,9 +5027,6 @@
     <t>hpflex</t>
   </si>
   <si>
-    <t>pathfndr-sr6</t>
-  </si>
-  <si>
     <t>hpflex-no-exp</t>
   </si>
   <si>
@@ -5039,9 +5036,6 @@
     <t>noflex</t>
   </si>
   <si>
-    <t>pathfndr-sr7</t>
-  </si>
-  <si>
     <t>noflex-no-exp</t>
   </si>
   <si>
@@ -5049,9 +5043,6 @@
   </si>
   <si>
     <t>bothflex</t>
-  </si>
-  <si>
-    <t>pathfndr-sr8</t>
   </si>
   <si>
     <t>bothflex-no-exp</t>
@@ -5091,7 +5082,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5161,6 +5152,12 @@
       <color rgb="FFA5D6FF"/>
       <name val="Menlo"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -16050,50 +16047,50 @@
         <v>1656</v>
       </c>
       <c r="B75" t="s">
-        <v>1657</v>
+        <v>1652</v>
       </c>
       <c r="C75" t="s">
         <v>1653</v>
       </c>
       <c r="D75" t="s">
+        <v>1657</v>
+      </c>
+      <c r="E75" t="s">
         <v>1658</v>
-      </c>
-      <c r="E75" t="s">
-        <v>1659</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>1660</v>
+        <v>1659</v>
       </c>
       <c r="B76" t="s">
-        <v>1661</v>
+        <v>1652</v>
       </c>
       <c r="C76" t="s">
         <v>1653</v>
       </c>
       <c r="D76" t="s">
-        <v>1662</v>
+        <v>1660</v>
       </c>
       <c r="E76" t="s">
-        <v>1663</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>1664</v>
+        <v>1662</v>
       </c>
       <c r="B77" t="s">
-        <v>1665</v>
+        <v>1652</v>
       </c>
       <c r="C77" t="s">
         <v>1653</v>
       </c>
       <c r="D77" t="s">
-        <v>1666</v>
+        <v>1663</v>
       </c>
       <c r="E77" t="s">
-        <v>1667</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
@@ -16104,13 +16101,13 @@
         <v>1652</v>
       </c>
       <c r="C78" t="s">
-        <v>1668</v>
+        <v>1665</v>
       </c>
       <c r="D78" t="s">
-        <v>1669</v>
+        <v>1666</v>
       </c>
       <c r="E78" t="s">
-        <v>1670</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
@@ -16118,53 +16115,54 @@
         <v>1656</v>
       </c>
       <c r="B79" t="s">
-        <v>1657</v>
+        <v>1652</v>
       </c>
       <c r="C79" t="s">
+        <v>1665</v>
+      </c>
+      <c r="D79" t="s">
         <v>1668</v>
       </c>
-      <c r="D79" t="s">
-        <v>1671</v>
-      </c>
       <c r="E79" t="s">
-        <v>1672</v>
+        <v>1669</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>1660</v>
+        <v>1659</v>
       </c>
       <c r="B80" t="s">
-        <v>1661</v>
+        <v>1652</v>
       </c>
       <c r="C80" t="s">
-        <v>1668</v>
+        <v>1665</v>
       </c>
       <c r="D80" t="s">
-        <v>1673</v>
+        <v>1670</v>
       </c>
       <c r="E80" t="s">
-        <v>1674</v>
+        <v>1671</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>1664</v>
+        <v>1662</v>
       </c>
       <c r="B81" t="s">
+        <v>1652</v>
+      </c>
+      <c r="C81" t="s">
         <v>1665</v>
       </c>
-      <c r="C81" t="s">
-        <v>1668</v>
-      </c>
       <c r="D81" t="s">
-        <v>1675</v>
+        <v>1672</v>
       </c>
       <c r="E81" t="s">
-        <v>1676</v>
+        <v>1673</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>